<commit_message>
Complete information engineering first-pass profiles and add evidence-gated mentor navigation
</commit_message>
<xml_diff>
--- a/site/exports/hit-computing.xlsx
+++ b/site/exports/hit-computing.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Rf587c0b1fccb4ac4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="R17200c637f9c4d8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="R8a1c6f0242714d8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="R09fcbdbf384e4c56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="Rf4a9629e1219497b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Rb8022c80a87c4012"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="Rdc0e8fd0da564b5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="Rea955dab63b84e7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="R879c6b3ec6af4f56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="R2a994fccef24495e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,6 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+  </x:numFmts>
   <x:fonts count="3">
     <x:font>
       <x:sz val="11"/>
@@ -58,13 +61,21 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="14">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -186,7 +197,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T0_4" displayName="T0_4" ref="A1:E5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T0_4" displayName="T0_4" ref="A1:E7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="来源ID"/>
@@ -403,78 +414,78 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+      <x:c r="A1" s="9" t="str">
         <x:v>姓名</x:v>
       </x:c>
-      <x:c r="B1" s="5" t="str">
+      <x:c r="B1" s="9" t="str">
         <x:v>校区</x:v>
       </x:c>
-      <x:c r="C1" s="5" t="str">
+      <x:c r="C1" s="9" t="str">
         <x:v>院系</x:v>
       </x:c>
-      <x:c r="D1" s="5" t="str">
+      <x:c r="D1" s="9" t="str">
         <x:v>官方主页</x:v>
       </x:c>
-      <x:c r="E1" s="5" t="str">
+      <x:c r="E1" s="9" t="str">
         <x:v>核对日期</x:v>
       </x:c>
-      <x:c r="F1" s="5" t="str">
+      <x:c r="F1" s="9" t="str">
         <x:v>缺项与冲突</x:v>
       </x:c>
-      <x:c r="G1" s="5" t="str">
+      <x:c r="G1" s="9" t="str">
         <x:v>范围</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="64" customHeight="1">
-      <x:c r="A2" s="3" t="str">
+      <x:c r="A2" s="6" t="str">
         <x:v>赵铁军</x:v>
       </x:c>
-      <x:c r="B2" s="3" t="str">
+      <x:c r="B2" s="6" t="str">
         <x:v>哈尔滨</x:v>
       </x:c>
-      <x:c r="C2" s="3" t="str">
+      <x:c r="C2" s="6" t="str">
         <x:v>计算学部</x:v>
       </x:c>
-      <x:c r="D2" s="3" t="str">
+      <x:c r="D2" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhaotiejun</x:v>
       </x:c>
-      <x:c r="E2" s="3" t="str">
-        <x:v>2026-10-23</x:v>
-      </x:c>
-      <x:c r="F2" s="3" t="str">
+      <x:c r="E2" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F2" s="6" t="str">
         <x:v>样本记录，不代表该院系全体教师；只收录已核实公开信息。；各学历阶段导师未在本次所核官方页面中找到明确证据。；主页列当前任职，尚未以人事信息独立核实退休或返聘状态。</x:v>
       </x:c>
-      <x:c r="G2" s="3" t="str">
+      <x:c r="G2" s="6" t="str">
         <x:v>分批核实资料，不是完整名录</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="64" customHeight="1">
-      <x:c r="A3" s="3" t="str">
+      <x:c r="A3" s="6" t="str">
         <x:v>丁效</x:v>
       </x:c>
-      <x:c r="B3" s="3" t="str">
+      <x:c r="B3" s="6" t="str">
         <x:v>哈尔滨</x:v>
       </x:c>
-      <x:c r="C3" s="3" t="str">
+      <x:c r="C3" s="6" t="str">
         <x:v>计算学部</x:v>
       </x:c>
-      <x:c r="D3" s="3" t="str">
+      <x:c r="D3" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/xiaoding</x:v>
       </x:c>
-      <x:c r="E3" s="3" t="str">
-        <x:v>2026-10-23</x:v>
-      </x:c>
-      <x:c r="F3" s="3" t="str">
+      <x:c r="E3" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F3" s="6" t="str">
         <x:v>样本记录，不代表该院系全体教师；只收录已核实公开信息。；各阶段导师未核实；不以论文合作作者反推导师。；官方中文正文列教授，英文正文列 Researcher，页头也有差异；职称需人工复核。</x:v>
       </x:c>
-      <x:c r="G3" s="3" t="str">
+      <x:c r="G3" s="6" t="str">
         <x:v>分批核实资料，不是完整名录</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0533408a9d8942ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4c1ccc48cf44427"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -503,402 +514,402 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+      <x:c r="A1" s="9" t="str">
         <x:v>姓名</x:v>
       </x:c>
-      <x:c r="B1" s="5" t="str">
+      <x:c r="B1" s="9" t="str">
         <x:v>事件类型</x:v>
       </x:c>
-      <x:c r="C1" s="5" t="str">
+      <x:c r="C1" s="9" t="str">
         <x:v>阶段/职位</x:v>
       </x:c>
-      <x:c r="D1" s="5" t="str">
+      <x:c r="D1" s="9" t="str">
         <x:v>机构</x:v>
       </x:c>
-      <x:c r="E1" s="5" t="str">
+      <x:c r="E1" s="9" t="str">
         <x:v>开始</x:v>
       </x:c>
-      <x:c r="F1" s="5" t="str">
+      <x:c r="F1" s="9" t="str">
         <x:v>结束</x:v>
       </x:c>
-      <x:c r="G1" s="5" t="str">
+      <x:c r="G1" s="9" t="str">
         <x:v>专业</x:v>
       </x:c>
-      <x:c r="H1" s="5" t="str">
+      <x:c r="H1" s="9" t="str">
         <x:v>国家</x:v>
       </x:c>
-      <x:c r="I1" s="5" t="str">
+      <x:c r="I1" s="9" t="str">
         <x:v>地区</x:v>
       </x:c>
-      <x:c r="J1" s="5" t="str">
+      <x:c r="J1" s="9" t="str">
         <x:v>洲</x:v>
       </x:c>
-      <x:c r="K1" s="5" t="str">
+      <x:c r="K1" s="9" t="str">
         <x:v>历史985分类</x:v>
       </x:c>
-      <x:c r="L1" s="5" t="str">
+      <x:c r="L1" s="9" t="str">
         <x:v>确证授位</x:v>
       </x:c>
-      <x:c r="M1" s="5" t="str">
+      <x:c r="M1" s="9" t="str">
         <x:v>授位日期</x:v>
       </x:c>
-      <x:c r="N1" s="5" t="str">
+      <x:c r="N1" s="9" t="str">
         <x:v>授位来源</x:v>
       </x:c>
-      <x:c r="O1" s="5" t="str">
+      <x:c r="O1" s="9" t="str">
         <x:v>备注及冲突</x:v>
       </x:c>
-      <x:c r="P1" s="5" t="str">
+      <x:c r="P1" s="9" t="str">
         <x:v>地域口径</x:v>
       </x:c>
-      <x:c r="Q1" s="5" t="str">
+      <x:c r="Q1" s="9" t="str">
         <x:v>来源</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="64" customHeight="1">
-      <x:c r="A2" s="3" t="str">
+      <x:c r="A2" s="6" t="str">
         <x:v>赵铁军</x:v>
       </x:c>
-      <x:c r="B2" s="3" t="str">
+      <x:c r="B2" s="6" t="str">
         <x:v>degree</x:v>
       </x:c>
-      <x:c r="C2" s="3" t="str">
+      <x:c r="C2" s="6" t="str">
         <x:v>学士</x:v>
       </x:c>
-      <x:c r="D2" s="3" t="str">
+      <x:c r="D2" s="6" t="str">
         <x:v>哈尔滨工业大学</x:v>
       </x:c>
-      <x:c r="E2" s="3" t="str">
+      <x:c r="E2" s="6" t="str">
         <x:v>1980</x:v>
       </x:c>
-      <x:c r="F2" s="3" t="str">
+      <x:c r="F2" s="6" t="str">
         <x:v>1984</x:v>
       </x:c>
-      <x:c r="G2" s="3" t="str">
+      <x:c r="G2" s="6" t="str">
         <x:v>计算机专业</x:v>
       </x:c>
-      <x:c r="H2" s="3" t="str">
+      <x:c r="H2" s="6" t="str">
         <x:v>中国</x:v>
       </x:c>
-      <x:c r="I2" s="3" t="str">
+      <x:c r="I2" s="6" t="str">
         <x:v>中国内地</x:v>
       </x:c>
-      <x:c r="J2" s="3" t="str">
+      <x:c r="J2" s="6" t="str">
         <x:v>亚洲</x:v>
       </x:c>
-      <x:c r="K2" s="3" t="str">
+      <x:c r="K2" s="6" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="L2" s="9" t="b">
+      <x:c r="L2" s="13" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="M2" s="3" t="str"/>
-      <x:c r="N2" s="3" t="str"/>
-      <x:c r="O2" s="3" t="str"/>
-      <x:c r="P2" s="3" t="str">
+      <x:c r="M2" s="7" t="str"/>
+      <x:c r="N2" s="6" t="str"/>
+      <x:c r="O2" s="6" t="str"/>
+      <x:c r="P2" s="6" t="str">
         <x:v>院校所在地标准化，不代表个人国籍或全部实际学习地点；中国香港单列，不归为国外。</x:v>
       </x:c>
-      <x:c r="Q2" s="3" t="str">
+      <x:c r="Q2" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhaotiejun</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="64" customHeight="1">
-      <x:c r="A3" s="3" t="str">
+      <x:c r="A3" s="6" t="str">
         <x:v>赵铁军</x:v>
       </x:c>
-      <x:c r="B3" s="3" t="str">
+      <x:c r="B3" s="6" t="str">
         <x:v>degree</x:v>
       </x:c>
-      <x:c r="C3" s="3" t="str">
+      <x:c r="C3" s="6" t="str">
         <x:v>硕士</x:v>
       </x:c>
-      <x:c r="D3" s="3" t="str">
+      <x:c r="D3" s="6" t="str">
         <x:v>哈尔滨工业大学</x:v>
       </x:c>
-      <x:c r="E3" s="3" t="str">
+      <x:c r="E3" s="6" t="str">
         <x:v>1987</x:v>
       </x:c>
-      <x:c r="F3" s="3" t="str">
+      <x:c r="F3" s="6" t="str">
         <x:v>1990</x:v>
       </x:c>
-      <x:c r="G3" s="3" t="str">
+      <x:c r="G3" s="6" t="str">
         <x:v>计算机系（专业名称未细分）</x:v>
       </x:c>
-      <x:c r="H3" s="3" t="str">
+      <x:c r="H3" s="6" t="str">
         <x:v>中国</x:v>
       </x:c>
-      <x:c r="I3" s="3" t="str">
+      <x:c r="I3" s="6" t="str">
         <x:v>中国内地</x:v>
       </x:c>
-      <x:c r="J3" s="3" t="str">
+      <x:c r="J3" s="6" t="str">
         <x:v>亚洲</x:v>
       </x:c>
-      <x:c r="K3" s="3" t="str">
+      <x:c r="K3" s="6" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="L3" s="9" t="b">
+      <x:c r="L3" s="13" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="M3" s="3" t="str"/>
-      <x:c r="N3" s="3" t="str"/>
-      <x:c r="O3" s="3" t="str"/>
-      <x:c r="P3" s="3" t="str">
+      <x:c r="M3" s="7" t="str"/>
+      <x:c r="N3" s="6" t="str"/>
+      <x:c r="O3" s="6" t="str"/>
+      <x:c r="P3" s="6" t="str">
         <x:v>院校所在地标准化，不代表个人国籍或全部实际学习地点；中国香港单列，不归为国外。</x:v>
       </x:c>
-      <x:c r="Q3" s="3" t="str">
+      <x:c r="Q3" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhaotiejun</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="64" customHeight="1">
-      <x:c r="A4" s="3" t="str">
+      <x:c r="A4" s="6" t="str">
         <x:v>赵铁军</x:v>
       </x:c>
-      <x:c r="B4" s="3" t="str">
+      <x:c r="B4" s="6" t="str">
         <x:v>degree</x:v>
       </x:c>
-      <x:c r="C4" s="3" t="str">
+      <x:c r="C4" s="6" t="str">
         <x:v>博士</x:v>
       </x:c>
-      <x:c r="D4" s="3" t="str">
+      <x:c r="D4" s="6" t="str">
         <x:v>哈尔滨工业大学</x:v>
       </x:c>
-      <x:c r="E4" s="3" t="str">
+      <x:c r="E4" s="6" t="str">
         <x:v>1994</x:v>
       </x:c>
-      <x:c r="F4" s="3" t="str">
+      <x:c r="F4" s="6" t="str">
         <x:v>1997</x:v>
       </x:c>
-      <x:c r="G4" s="3" t="str">
+      <x:c r="G4" s="6" t="str">
         <x:v>计算机系（在职攻读）</x:v>
       </x:c>
-      <x:c r="H4" s="3" t="str">
+      <x:c r="H4" s="6" t="str">
         <x:v>中国</x:v>
       </x:c>
-      <x:c r="I4" s="3" t="str">
+      <x:c r="I4" s="6" t="str">
         <x:v>中国内地</x:v>
       </x:c>
-      <x:c r="J4" s="3" t="str">
+      <x:c r="J4" s="6" t="str">
         <x:v>亚洲</x:v>
       </x:c>
-      <x:c r="K4" s="3" t="str">
+      <x:c r="K4" s="6" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="L4" s="9" t="b">
+      <x:c r="L4" s="13" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="M4" s="3" t="str"/>
-      <x:c r="N4" s="3" t="str"/>
-      <x:c r="O4" s="3" t="str"/>
-      <x:c r="P4" s="3" t="str">
+      <x:c r="M4" s="7" t="str"/>
+      <x:c r="N4" s="6" t="str"/>
+      <x:c r="O4" s="6" t="str"/>
+      <x:c r="P4" s="6" t="str">
         <x:v>院校所在地标准化，不代表个人国籍或全部实际学习地点；中国香港单列，不归为国外。</x:v>
       </x:c>
-      <x:c r="Q4" s="3" t="str">
+      <x:c r="Q4" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhaotiejun</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="64" customHeight="1">
-      <x:c r="A5" s="3" t="str">
+      <x:c r="A5" s="6" t="str">
         <x:v>赵铁军</x:v>
       </x:c>
-      <x:c r="B5" s="3" t="str">
+      <x:c r="B5" s="6" t="str">
         <x:v>employment</x:v>
       </x:c>
-      <x:c r="C5" s="3" t="str">
+      <x:c r="C5" s="6" t="str">
         <x:v>教授、博士生导师</x:v>
       </x:c>
-      <x:c r="D5" s="3" t="str">
+      <x:c r="D5" s="6" t="str">
         <x:v>哈尔滨工业大学</x:v>
       </x:c>
-      <x:c r="E5" s="3" t="str"/>
-      <x:c r="F5" s="3" t="str"/>
-      <x:c r="G5" s="3" t="str"/>
-      <x:c r="H5" s="3" t="str"/>
-      <x:c r="I5" s="3" t="str"/>
-      <x:c r="J5" s="3" t="str"/>
-      <x:c r="K5" s="3" t="str"/>
-      <x:c r="L5" s="3" t="str"/>
-      <x:c r="M5" s="3" t="str"/>
-      <x:c r="N5" s="3" t="str"/>
-      <x:c r="O5" s="3" t="str"/>
-      <x:c r="P5" s="3" t="str"/>
-      <x:c r="Q5" s="3" t="str">
+      <x:c r="E5" s="6" t="str"/>
+      <x:c r="F5" s="6" t="str"/>
+      <x:c r="G5" s="6" t="str"/>
+      <x:c r="H5" s="6" t="str"/>
+      <x:c r="I5" s="6" t="str"/>
+      <x:c r="J5" s="6" t="str"/>
+      <x:c r="K5" s="6" t="str"/>
+      <x:c r="L5" s="6" t="str"/>
+      <x:c r="M5" s="7" t="str"/>
+      <x:c r="N5" s="6" t="str"/>
+      <x:c r="O5" s="6" t="str"/>
+      <x:c r="P5" s="6" t="str"/>
+      <x:c r="Q5" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhaotiejun</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="64" customHeight="1">
-      <x:c r="A6" s="3" t="str">
+      <x:c r="A6" s="6" t="str">
         <x:v>丁效</x:v>
       </x:c>
-      <x:c r="B6" s="3" t="str">
+      <x:c r="B6" s="6" t="str">
         <x:v>degree</x:v>
       </x:c>
-      <x:c r="C6" s="3" t="str">
+      <x:c r="C6" s="6" t="str">
         <x:v>本科</x:v>
       </x:c>
-      <x:c r="D6" s="3" t="str">
+      <x:c r="D6" s="6" t="str">
         <x:v>哈尔滨工业大学</x:v>
       </x:c>
-      <x:c r="E6" s="3" t="str">
+      <x:c r="E6" s="6" t="str">
         <x:v>2005-09</x:v>
       </x:c>
-      <x:c r="F6" s="3" t="str">
+      <x:c r="F6" s="6" t="str">
         <x:v>2009-07</x:v>
       </x:c>
-      <x:c r="G6" s="3" t="str">
+      <x:c r="G6" s="6" t="str">
         <x:v>计算机科学与技术</x:v>
       </x:c>
-      <x:c r="H6" s="3" t="str">
+      <x:c r="H6" s="6" t="str">
         <x:v>中国</x:v>
       </x:c>
-      <x:c r="I6" s="3" t="str">
+      <x:c r="I6" s="6" t="str">
         <x:v>中国内地</x:v>
       </x:c>
-      <x:c r="J6" s="3" t="str">
+      <x:c r="J6" s="6" t="str">
         <x:v>亚洲</x:v>
       </x:c>
-      <x:c r="K6" s="3" t="str">
+      <x:c r="K6" s="6" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="L6" s="9" t="b">
+      <x:c r="L6" s="13" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="M6" s="3" t="str"/>
-      <x:c r="N6" s="3" t="str"/>
-      <x:c r="O6" s="3" t="str"/>
-      <x:c r="P6" s="3" t="str">
+      <x:c r="M6" s="7" t="str"/>
+      <x:c r="N6" s="6" t="str"/>
+      <x:c r="O6" s="6" t="str"/>
+      <x:c r="P6" s="6" t="str">
         <x:v>院校所在地标准化，不代表个人国籍或全部实际学习地点；中国香港单列，不归为国外。</x:v>
       </x:c>
-      <x:c r="Q6" s="3" t="str">
+      <x:c r="Q6" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/xiaoding</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="64" customHeight="1">
-      <x:c r="A7" s="3" t="str">
+      <x:c r="A7" s="6" t="str">
         <x:v>丁效</x:v>
       </x:c>
-      <x:c r="B7" s="3" t="str">
+      <x:c r="B7" s="6" t="str">
         <x:v>degree</x:v>
       </x:c>
-      <x:c r="C7" s="3" t="str">
+      <x:c r="C7" s="6" t="str">
         <x:v>硕士</x:v>
       </x:c>
-      <x:c r="D7" s="3" t="str">
+      <x:c r="D7" s="6" t="str">
         <x:v>哈尔滨工业大学</x:v>
       </x:c>
-      <x:c r="E7" s="3" t="str">
+      <x:c r="E7" s="6" t="str">
         <x:v>2009-09</x:v>
       </x:c>
-      <x:c r="F7" s="3" t="str">
+      <x:c r="F7" s="6" t="str">
         <x:v>2011-07</x:v>
       </x:c>
-      <x:c r="G7" s="3" t="str">
+      <x:c r="G7" s="6" t="str">
         <x:v>计算机科学与技术</x:v>
       </x:c>
-      <x:c r="H7" s="3" t="str">
+      <x:c r="H7" s="6" t="str">
         <x:v>中国</x:v>
       </x:c>
-      <x:c r="I7" s="3" t="str">
+      <x:c r="I7" s="6" t="str">
         <x:v>中国内地</x:v>
       </x:c>
-      <x:c r="J7" s="3" t="str">
+      <x:c r="J7" s="6" t="str">
         <x:v>亚洲</x:v>
       </x:c>
-      <x:c r="K7" s="3" t="str">
+      <x:c r="K7" s="6" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="L7" s="9" t="b">
+      <x:c r="L7" s="13" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="M7" s="3" t="str"/>
-      <x:c r="N7" s="3" t="str"/>
-      <x:c r="O7" s="3" t="str"/>
-      <x:c r="P7" s="3" t="str">
+      <x:c r="M7" s="7" t="str"/>
+      <x:c r="N7" s="6" t="str"/>
+      <x:c r="O7" s="6" t="str"/>
+      <x:c r="P7" s="6" t="str">
         <x:v>院校所在地标准化，不代表个人国籍或全部实际学习地点；中国香港单列，不归为国外。</x:v>
       </x:c>
-      <x:c r="Q7" s="3" t="str">
+      <x:c r="Q7" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/xiaoding</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="64" customHeight="1">
-      <x:c r="A8" s="3" t="str">
+      <x:c r="A8" s="6" t="str">
         <x:v>丁效</x:v>
       </x:c>
-      <x:c r="B8" s="3" t="str">
+      <x:c r="B8" s="6" t="str">
         <x:v>degree</x:v>
       </x:c>
-      <x:c r="C8" s="3" t="str">
+      <x:c r="C8" s="6" t="str">
         <x:v>博士</x:v>
       </x:c>
-      <x:c r="D8" s="3" t="str">
+      <x:c r="D8" s="6" t="str">
         <x:v>哈尔滨工业大学</x:v>
       </x:c>
-      <x:c r="E8" s="3" t="str">
+      <x:c r="E8" s="6" t="str">
         <x:v>2011-09</x:v>
       </x:c>
-      <x:c r="F8" s="3" t="str">
+      <x:c r="F8" s="6" t="str">
         <x:v>2016-06</x:v>
       </x:c>
-      <x:c r="G8" s="3" t="str">
+      <x:c r="G8" s="6" t="str">
         <x:v>计算机应用技术</x:v>
       </x:c>
-      <x:c r="H8" s="3" t="str">
+      <x:c r="H8" s="6" t="str">
         <x:v>中国</x:v>
       </x:c>
-      <x:c r="I8" s="3" t="str">
+      <x:c r="I8" s="6" t="str">
         <x:v>中国内地</x:v>
       </x:c>
-      <x:c r="J8" s="3" t="str">
+      <x:c r="J8" s="6" t="str">
         <x:v>亚洲</x:v>
       </x:c>
-      <x:c r="K8" s="3" t="str">
+      <x:c r="K8" s="6" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="L8" s="9" t="b">
+      <x:c r="L8" s="13" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="M8" s="3" t="str"/>
-      <x:c r="N8" s="3" t="str"/>
-      <x:c r="O8" s="3" t="str"/>
-      <x:c r="P8" s="3" t="str">
+      <x:c r="M8" s="7" t="str"/>
+      <x:c r="N8" s="6" t="str"/>
+      <x:c r="O8" s="6" t="str"/>
+      <x:c r="P8" s="6" t="str">
         <x:v>院校所在地标准化，不代表个人国籍或全部实际学习地点；中国香港单列，不归为国外。</x:v>
       </x:c>
-      <x:c r="Q8" s="3" t="str">
+      <x:c r="Q8" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/xiaoding</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="64" customHeight="1">
-      <x:c r="A9" s="3" t="str">
+      <x:c r="A9" s="6" t="str">
         <x:v>丁效</x:v>
       </x:c>
-      <x:c r="B9" s="3" t="str">
+      <x:c r="B9" s="6" t="str">
         <x:v>employment</x:v>
       </x:c>
-      <x:c r="C9" s="3" t="str">
+      <x:c r="C9" s="6" t="str">
         <x:v>教授、博士生导师（正文）；页头为研究员/博导</x:v>
       </x:c>
-      <x:c r="D9" s="3" t="str">
+      <x:c r="D9" s="6" t="str">
         <x:v>哈尔滨工业大学</x:v>
       </x:c>
-      <x:c r="E9" s="3" t="str"/>
-      <x:c r="F9" s="3" t="str"/>
-      <x:c r="G9" s="3" t="str"/>
-      <x:c r="H9" s="3" t="str"/>
-      <x:c r="I9" s="3" t="str"/>
-      <x:c r="J9" s="3" t="str"/>
-      <x:c r="K9" s="3" t="str"/>
-      <x:c r="L9" s="3" t="str"/>
-      <x:c r="M9" s="3" t="str"/>
-      <x:c r="N9" s="3" t="str"/>
-      <x:c r="O9" s="3" t="str"/>
-      <x:c r="P9" s="3" t="str"/>
-      <x:c r="Q9" s="3" t="str">
+      <x:c r="E9" s="6" t="str"/>
+      <x:c r="F9" s="6" t="str"/>
+      <x:c r="G9" s="6" t="str"/>
+      <x:c r="H9" s="6" t="str"/>
+      <x:c r="I9" s="6" t="str"/>
+      <x:c r="J9" s="6" t="str"/>
+      <x:c r="K9" s="6" t="str"/>
+      <x:c r="L9" s="6" t="str"/>
+      <x:c r="M9" s="7" t="str"/>
+      <x:c r="N9" s="6" t="str"/>
+      <x:c r="O9" s="6" t="str"/>
+      <x:c r="P9" s="6" t="str"/>
+      <x:c r="Q9" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/xiaoding</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad3ea88bc4ca496f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55aa6f0834d3414c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -920,34 +931,34 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+      <x:c r="A1" s="9" t="str">
         <x:v>姓名</x:v>
       </x:c>
-      <x:c r="B1" s="5" t="str">
+      <x:c r="B1" s="9" t="str">
         <x:v>导师姓名</x:v>
       </x:c>
-      <x:c r="C1" s="5" t="str">
+      <x:c r="C1" s="9" t="str">
         <x:v>关系类型</x:v>
       </x:c>
-      <x:c r="D1" s="5" t="str">
+      <x:c r="D1" s="9" t="str">
         <x:v>阶段</x:v>
       </x:c>
-      <x:c r="E1" s="5" t="str">
+      <x:c r="E1" s="9" t="str">
         <x:v>简介</x:v>
       </x:c>
-      <x:c r="F1" s="5" t="str">
+      <x:c r="F1" s="9" t="str">
         <x:v>在职状态</x:v>
       </x:c>
-      <x:c r="G1" s="5" t="str">
+      <x:c r="G1" s="9" t="str">
         <x:v>状态说明</x:v>
       </x:c>
-      <x:c r="H1" s="5" t="str">
+      <x:c r="H1" s="9" t="str">
         <x:v>已核在职主页</x:v>
       </x:c>
-      <x:c r="I1" s="5" t="str">
+      <x:c r="I1" s="9" t="str">
         <x:v>关系来源</x:v>
       </x:c>
-      <x:c r="J1" s="5" t="str">
+      <x:c r="J1" s="9" t="str">
         <x:v>任职来源</x:v>
       </x:c>
     </x:row>
@@ -973,97 +984,97 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+      <x:c r="A1" s="9" t="str">
         <x:v>姓名</x:v>
       </x:c>
-      <x:c r="B1" s="5" t="str">
+      <x:c r="B1" s="9" t="str">
         <x:v>标题</x:v>
       </x:c>
-      <x:c r="C1" s="5" t="str">
+      <x:c r="C1" s="9" t="str">
         <x:v>年份</x:v>
       </x:c>
-      <x:c r="D1" s="5" t="str">
+      <x:c r="D1" s="9" t="str">
         <x:v>DOI</x:v>
       </x:c>
-      <x:c r="E1" s="5" t="str">
+      <x:c r="E1" s="9" t="str">
         <x:v>链接</x:v>
       </x:c>
-      <x:c r="F1" s="5" t="str">
+      <x:c r="F1" s="9" t="str">
         <x:v>类型</x:v>
       </x:c>
-      <x:c r="G1" s="5" t="str">
+      <x:c r="G1" s="9" t="str">
         <x:v>收录来源</x:v>
       </x:c>
-      <x:c r="H1" s="5" t="str">
+      <x:c r="H1" s="9" t="str">
         <x:v>作者归属依据</x:v>
       </x:c>
-      <x:c r="I1" s="5" t="str">
+      <x:c r="I1" s="9" t="str">
         <x:v>链接核验范围</x:v>
       </x:c>
-      <x:c r="J1" s="5" t="str">
+      <x:c r="J1" s="9" t="str">
         <x:v>备注</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="64" customHeight="1">
-      <x:c r="A2" s="3" t="str">
+      <x:c r="A2" s="6" t="str">
         <x:v>赵铁军</x:v>
       </x:c>
-      <x:c r="B2" s="3" t="str">
+      <x:c r="B2" s="6" t="str">
         <x:v>CoLaDa: A Collaborative Label Denoising Framework for Cross-lingual Named Entity Recognition</x:v>
       </x:c>
-      <x:c r="C2" s="3" t="n">
+      <x:c r="C2" s="6" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="D2" s="3" t="str">
+      <x:c r="D2" s="6" t="str">
         <x:v>10.18653/v1/2023.acl-long.330</x:v>
       </x:c>
-      <x:c r="E2" s="3" t="str">
+      <x:c r="E2" s="6" t="str">
         <x:v>https://aclanthology.org/2023.acl-long.330/</x:v>
       </x:c>
-      <x:c r="F2" s="3" t="str">
+      <x:c r="F2" s="6" t="str">
         <x:v>conference_paper</x:v>
       </x:c>
-      <x:c r="G2" s="3" t="str">
+      <x:c r="G2" s="6" t="str">
         <x:v>https://aclanthology.org/2023.acl-long.330/</x:v>
       </x:c>
-      <x:c r="H2" s="3" t="str">
+      <x:c r="H2" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhaotiejun</x:v>
       </x:c>
-      <x:c r="I2" s="3" t="str"/>
-      <x:c r="J2" s="3" t="str"/>
+      <x:c r="I2" s="6" t="str"/>
+      <x:c r="J2" s="6" t="str"/>
     </x:row>
     <x:row r="3" ht="64" customHeight="1">
-      <x:c r="A3" s="3" t="str">
+      <x:c r="A3" s="6" t="str">
         <x:v>丁效</x:v>
       </x:c>
-      <x:c r="B3" s="3" t="str">
+      <x:c r="B3" s="6" t="str">
         <x:v>TinyJudge: Unverifiable Constraint Alignment via Lightweight Specialist Ensembles</x:v>
       </x:c>
-      <x:c r="C3" s="3" t="n">
+      <x:c r="C3" s="6" t="n">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="D3" s="3" t="str"/>
-      <x:c r="E3" s="3" t="str">
+      <x:c r="D3" s="6" t="str"/>
+      <x:c r="E3" s="6" t="str">
         <x:v>https://aclanthology.org/2026.acl-long.1204.pdf</x:v>
       </x:c>
-      <x:c r="F3" s="3" t="str">
+      <x:c r="F3" s="6" t="str">
         <x:v>conference_paper</x:v>
       </x:c>
-      <x:c r="G3" s="3" t="str">
+      <x:c r="G3" s="6" t="str">
         <x:v>https://aclanthology.org/2026.acl-long.1204.pdf</x:v>
       </x:c>
-      <x:c r="H3" s="3" t="str">
+      <x:c r="H3" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/xiaoding</x:v>
       </x:c>
-      <x:c r="I3" s="3" t="str">
+      <x:c r="I3" s="6" t="str">
         <x:v>官网列示与ACL出版方PDF交叉核验；仅链接不复制论文</x:v>
       </x:c>
-      <x:c r="J3" s="3" t="str"/>
+      <x:c r="J3" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61420df7570947ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbe1098821cb4b57"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1080,94 +1091,128 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+      <x:c r="A1" s="9" t="str">
         <x:v>姓名</x:v>
       </x:c>
-      <x:c r="B1" s="5" t="str">
+      <x:c r="B1" s="9" t="str">
         <x:v>来源ID</x:v>
       </x:c>
-      <x:c r="C1" s="5" t="str">
+      <x:c r="C1" s="9" t="str">
         <x:v>链接</x:v>
       </x:c>
-      <x:c r="D1" s="5" t="str">
+      <x:c r="D1" s="9" t="str">
         <x:v>核验方式</x:v>
       </x:c>
-      <x:c r="E1" s="5" t="str">
+      <x:c r="E1" s="9" t="str">
         <x:v>查阅日期</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="64" customHeight="1">
-      <x:c r="A2" s="3" t="str">
+      <x:c r="A2" s="6" t="str">
         <x:v>赵铁军</x:v>
       </x:c>
-      <x:c r="B2" s="3" t="str">
+      <x:c r="B2" s="6" t="str">
         <x:v>zhaotiejun-official</x:v>
       </x:c>
-      <x:c r="C2" s="3" t="str">
+      <x:c r="C2" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhaotiejun</x:v>
       </x:c>
-      <x:c r="D2" s="3" t="str">
+      <x:c r="D2" s="6" t="str">
         <x:v>official_page_public_body_fetched</x:v>
       </x:c>
-      <x:c r="E2" s="3" t="str">
-        <x:v>2026-10-23</x:v>
+      <x:c r="E2" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="64" customHeight="1">
-      <x:c r="A3" s="3" t="str">
+      <x:c r="A3" s="6" t="str">
         <x:v>赵铁军</x:v>
       </x:c>
-      <x:c r="B3" s="3" t="str">
+      <x:c r="B3" s="6" t="str">
         <x:v>hit-zhaotiejun-publication-1</x:v>
       </x:c>
-      <x:c r="C3" s="3" t="str">
+      <x:c r="C3" s="6" t="str">
         <x:v>https://aclanthology.org/2023.acl-long.330/</x:v>
       </x:c>
-      <x:c r="D3" s="3" t="str">
+      <x:c r="D3" s="6" t="str">
         <x:v>official_publisher_or_institution_metadata</x:v>
       </x:c>
-      <x:c r="E3" s="3" t="str">
-        <x:v>2026-10-23</x:v>
+      <x:c r="E3" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="64" customHeight="1">
-      <x:c r="A4" s="3" t="str">
+      <x:c r="A4" s="6" t="str">
         <x:v>丁效</x:v>
       </x:c>
-      <x:c r="B4" s="3" t="str">
+      <x:c r="B4" s="6" t="str">
         <x:v>xiaoding-official</x:v>
       </x:c>
-      <x:c r="C4" s="3" t="str">
+      <x:c r="C4" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/xiaoding</x:v>
       </x:c>
-      <x:c r="D4" s="3" t="str">
+      <x:c r="D4" s="6" t="str">
         <x:v>official_page_public_body_fetched</x:v>
       </x:c>
-      <x:c r="E4" s="3" t="str">
-        <x:v>2026-10-23</x:v>
+      <x:c r="E4" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="64" customHeight="1">
-      <x:c r="A5" s="3" t="str">
+      <x:c r="A5" s="6" t="str">
         <x:v>丁效</x:v>
       </x:c>
-      <x:c r="B5" s="3" t="str">
+      <x:c r="B5" s="6" t="str">
         <x:v>xiaoding-publication-1</x:v>
       </x:c>
-      <x:c r="C5" s="3" t="str">
+      <x:c r="C5" s="6" t="str">
         <x:v>https://aclanthology.org/2026.acl-long.1204.pdf</x:v>
       </x:c>
-      <x:c r="D5" s="3" t="str">
+      <x:c r="D5" s="6" t="str">
         <x:v>official_publisher_pdf_index</x:v>
       </x:c>
-      <x:c r="E5" s="3" t="str">
-        <x:v>2026-10-23</x:v>
+      <x:c r="E5" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="64" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>赵铁军</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>institution-classification-2</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="str">
+        <x:v>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="str">
+        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+      </x:c>
+      <x:c r="E6" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="64" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>丁效</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="str">
+        <x:v>institution-classification-2</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="str">
+        <x:v>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="str">
+        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+      </x:c>
+      <x:c r="E7" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f66076680b74ca1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55a953bec3f54050"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add reviewed Weihai profiles and preserve source identity and snapshot consistency
</commit_message>
<xml_diff>
--- a/site/exports/hit-computing.xlsx
+++ b/site/exports/hit-computing.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Rb8022c80a87c4012"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="Rdc0e8fd0da564b5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="Rea955dab63b84e7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="R879c6b3ec6af4f56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="R2a994fccef24495e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R64dbc204801945e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="R191dca1efd5e4b13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="R55e8f44ad435476b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="Rb376450334b04d54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="R7d5730aa7e7b467b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,8 +139,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T0_0" displayName="T0_0" ref="A1:G3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="7">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T0_0" displayName="T0_0" ref="A1:I3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="校区"/>
     <x:tableColumn id="3" name="院系"/>
@@ -148,6 +148,8 @@
     <x:tableColumn id="5" name="核对日期"/>
     <x:tableColumn id="6" name="缺项与冲突"/>
     <x:tableColumn id="7" name="范围"/>
+    <x:tableColumn id="8" name="主页可用性"/>
+    <x:tableColumn id="9" name="替代官方职业报道（非个人主页）"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -411,6 +413,8 @@
     <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="55" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="55" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="26" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -435,6 +439,12 @@
       <x:c r="G1" s="9" t="str">
         <x:v>范围</x:v>
       </x:c>
+      <x:c r="H1" s="9" t="str">
+        <x:v>主页可用性</x:v>
+      </x:c>
+      <x:c r="I1" s="9" t="str">
+        <x:v>替代官方职业报道（非个人主页）</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="64" customHeight="1">
       <x:c r="A2" s="6" t="str">
@@ -458,6 +468,10 @@
       <x:c r="G2" s="6" t="str">
         <x:v>分批核实资料，不是完整名录</x:v>
       </x:c>
+      <x:c r="H2" s="6" t="str">
+        <x:v>公开个人页（时效以核对日为准）</x:v>
+      </x:c>
+      <x:c r="I2" s="6" t="str"/>
     </x:row>
     <x:row r="3" ht="64" customHeight="1">
       <x:c r="A3" s="6" t="str">
@@ -481,11 +495,15 @@
       <x:c r="G3" s="6" t="str">
         <x:v>分批核实资料，不是完整名录</x:v>
       </x:c>
+      <x:c r="H3" s="6" t="str">
+        <x:v>公开个人页（时效以核对日为准）</x:v>
+      </x:c>
+      <x:c r="I3" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4c1ccc48cf44427"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba851e896b434e62"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -909,7 +927,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55aa6f0834d3414c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5612cb66e1b494a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1074,7 +1092,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbe1098821cb4b57"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0662f0b1e2bf434c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1212,7 +1230,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55a953bec3f54050"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c7757749c7e48fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add reviewed first samples from four universities and school-scoped navigation
</commit_message>
<xml_diff>
--- a/site/exports/hit-computing.xlsx
+++ b/site/exports/hit-computing.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R64dbc204801945e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="R191dca1efd5e4b13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="R55e8f44ad435476b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="Rb376450334b04d54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="R7d5730aa7e7b467b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Rb5f6df3c027a4baf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="R810450e7f16e4f92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="R66a5325d56084e9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="R322e7acbe1374bc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="R5cd3cdfddc8d4fc3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,8 +139,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T0_0" displayName="T0_0" ref="A1:I3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="9">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T0_0" displayName="T0_0" ref="A1:K3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="校区"/>
     <x:tableColumn id="3" name="院系"/>
@@ -150,14 +150,16 @@
     <x:tableColumn id="7" name="范围"/>
     <x:tableColumn id="8" name="主页可用性"/>
     <x:tableColumn id="9" name="替代官方职业报道（非个人主页）"/>
+    <x:tableColumn id="10" name="所属学校ID"/>
+    <x:tableColumn id="11" name="所属学校"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T0_1" displayName="T0_1" ref="A1:Q9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="17">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T0_1" displayName="T0_1" ref="A1:S9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="19">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="事件类型"/>
     <x:tableColumn id="3" name="阶段/职位"/>
@@ -175,14 +177,16 @@
     <x:tableColumn id="15" name="备注及冲突"/>
     <x:tableColumn id="16" name="地域口径"/>
     <x:tableColumn id="17" name="来源"/>
+    <x:tableColumn id="18" name="所属学校ID"/>
+    <x:tableColumn id="19" name="所属学校"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T0_3" displayName="T0_3" ref="A1:J3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="10">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T0_3" displayName="T0_3" ref="A1:L3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="12">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="标题"/>
     <x:tableColumn id="3" name="年份"/>
@@ -193,19 +197,23 @@
     <x:tableColumn id="8" name="作者归属依据"/>
     <x:tableColumn id="9" name="链接核验范围"/>
     <x:tableColumn id="10" name="备注"/>
+    <x:tableColumn id="11" name="所属学校ID"/>
+    <x:tableColumn id="12" name="所属学校"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T0_4" displayName="T0_4" ref="A1:E7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="5">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T0_4" displayName="T0_4" ref="A1:G7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="7">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="来源ID"/>
     <x:tableColumn id="3" name="链接"/>
     <x:tableColumn id="4" name="核验方式"/>
     <x:tableColumn id="5" name="查阅日期"/>
+    <x:tableColumn id="6" name="所属学校ID"/>
+    <x:tableColumn id="7" name="所属学校"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -415,6 +423,8 @@
     <x:col min="7" max="7" width="55" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="26" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="26" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="26" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -445,6 +455,12 @@
       <x:c r="I1" s="9" t="str">
         <x:v>替代官方职业报道（非个人主页）</x:v>
       </x:c>
+      <x:c r="J1" s="9" t="str">
+        <x:v>所属学校ID</x:v>
+      </x:c>
+      <x:c r="K1" s="9" t="str">
+        <x:v>所属学校</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="64" customHeight="1">
       <x:c r="A2" s="6" t="str">
@@ -472,6 +488,12 @@
         <x:v>公开个人页（时效以核对日为准）</x:v>
       </x:c>
       <x:c r="I2" s="6" t="str"/>
+      <x:c r="J2" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="K2" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="64" customHeight="1">
       <x:c r="A3" s="6" t="str">
@@ -499,11 +521,17 @@
         <x:v>公开个人页（时效以核对日为准）</x:v>
       </x:c>
       <x:c r="I3" s="6" t="str"/>
+      <x:c r="J3" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="K3" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba851e896b434e62"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67f1ed03a3ed496f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -529,6 +557,8 @@
     <x:col min="15" max="15" width="55" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="26" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="55" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="26" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -583,6 +613,12 @@
       <x:c r="Q1" s="9" t="str">
         <x:v>来源</x:v>
       </x:c>
+      <x:c r="R1" s="9" t="str">
+        <x:v>所属学校ID</x:v>
+      </x:c>
+      <x:c r="S1" s="9" t="str">
+        <x:v>所属学校</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="64" customHeight="1">
       <x:c r="A2" s="6" t="str">
@@ -630,6 +666,12 @@
       <x:c r="Q2" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhaotiejun</x:v>
       </x:c>
+      <x:c r="R2" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="S2" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="64" customHeight="1">
       <x:c r="A3" s="6" t="str">
@@ -677,6 +719,12 @@
       <x:c r="Q3" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhaotiejun</x:v>
       </x:c>
+      <x:c r="R3" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="S3" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="64" customHeight="1">
       <x:c r="A4" s="6" t="str">
@@ -723,6 +771,12 @@
       </x:c>
       <x:c r="Q4" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhaotiejun</x:v>
+      </x:c>
+      <x:c r="R4" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="S4" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="64" customHeight="1">
@@ -753,6 +807,12 @@
       <x:c r="Q5" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhaotiejun</x:v>
       </x:c>
+      <x:c r="R5" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="S5" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="64" customHeight="1">
       <x:c r="A6" s="6" t="str">
@@ -800,6 +860,12 @@
       <x:c r="Q6" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/xiaoding</x:v>
       </x:c>
+      <x:c r="R6" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="S6" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="64" customHeight="1">
       <x:c r="A7" s="6" t="str">
@@ -847,6 +913,12 @@
       <x:c r="Q7" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/xiaoding</x:v>
       </x:c>
+      <x:c r="R7" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="S7" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="64" customHeight="1">
       <x:c r="A8" s="6" t="str">
@@ -893,6 +965,12 @@
       </x:c>
       <x:c r="Q8" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/xiaoding</x:v>
+      </x:c>
+      <x:c r="R8" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="S8" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="64" customHeight="1">
@@ -923,11 +1001,17 @@
       <x:c r="Q9" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/xiaoding</x:v>
       </x:c>
+      <x:c r="R9" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="S9" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5612cb66e1b494a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra78d203bef6f435f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -946,6 +1030,8 @@
     <x:col min="8" max="8" width="26" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="55" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="55" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -978,6 +1064,12 @@
       </x:c>
       <x:c r="J1" s="9" t="str">
         <x:v>任职来源</x:v>
+      </x:c>
+      <x:c r="K1" s="9" t="str">
+        <x:v>所属学校ID</x:v>
+      </x:c>
+      <x:c r="L1" s="9" t="str">
+        <x:v>所属学校</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -999,6 +1091,8 @@
     <x:col min="8" max="8" width="26" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="55" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="55" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -1032,6 +1126,12 @@
       <x:c r="J1" s="9" t="str">
         <x:v>备注</x:v>
       </x:c>
+      <x:c r="K1" s="9" t="str">
+        <x:v>所属学校ID</x:v>
+      </x:c>
+      <x:c r="L1" s="9" t="str">
+        <x:v>所属学校</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="64" customHeight="1">
       <x:c r="A2" s="6" t="str">
@@ -1060,6 +1160,12 @@
       </x:c>
       <x:c r="I2" s="6" t="str"/>
       <x:c r="J2" s="6" t="str"/>
+      <x:c r="K2" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="L2" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="64" customHeight="1">
       <x:c r="A3" s="6" t="str">
@@ -1088,11 +1194,17 @@
         <x:v>官网列示与ACL出版方PDF交叉核验；仅链接不复制论文</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str"/>
+      <x:c r="K3" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="L3" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0662f0b1e2bf434c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe4b6bca69504821"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1106,6 +1218,8 @@
     <x:col min="3" max="3" width="55" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="26" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="26" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -1124,6 +1238,12 @@
       <x:c r="E1" s="9" t="str">
         <x:v>查阅日期</x:v>
       </x:c>
+      <x:c r="F1" s="9" t="str">
+        <x:v>所属学校ID</x:v>
+      </x:c>
+      <x:c r="G1" s="9" t="str">
+        <x:v>所属学校</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="64" customHeight="1">
       <x:c r="A2" s="6" t="str">
@@ -1141,6 +1261,12 @@
       <x:c r="E2" s="7" t="d">
         <x:v>2026-10-23T00:00:00.000Z</x:v>
       </x:c>
+      <x:c r="F2" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="G2" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="64" customHeight="1">
       <x:c r="A3" s="6" t="str">
@@ -1158,6 +1284,12 @@
       <x:c r="E3" s="7" t="d">
         <x:v>2026-10-23T00:00:00.000Z</x:v>
       </x:c>
+      <x:c r="F3" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="G3" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="64" customHeight="1">
       <x:c r="A4" s="6" t="str">
@@ -1175,6 +1307,12 @@
       <x:c r="E4" s="7" t="d">
         <x:v>2026-10-23T00:00:00.000Z</x:v>
       </x:c>
+      <x:c r="F4" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="G4" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="64" customHeight="1">
       <x:c r="A5" s="6" t="str">
@@ -1192,6 +1330,12 @@
       <x:c r="E5" s="7" t="d">
         <x:v>2026-10-23T00:00:00.000Z</x:v>
       </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="64" customHeight="1">
       <x:c r="A6" s="6" t="str">
@@ -1209,6 +1353,12 @@
       <x:c r="E6" s="7" t="d">
         <x:v>2026-10-23T00:00:00.000Z</x:v>
       </x:c>
+      <x:c r="F6" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="G6" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="64" customHeight="1">
       <x:c r="A7" s="6" t="str">
@@ -1226,11 +1376,17 @@
       <x:c r="E7" s="7" t="d">
         <x:v>2026-10-23T00:00:00.000Z</x:v>
       </x:c>
+      <x:c r="F7" s="6" t="str">
+        <x:v>hit</x:v>
+      </x:c>
+      <x:c r="G7" s="6" t="str">
+        <x:v>哈尔滨工业大学</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c7757749c7e48fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b834b4a49284b1d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>